<commit_message>
Update investor workbook, sync data, and add Michael Gentile photo
Refresh GS-Investors.xlsx and regenerated investors.json (87 position rows). Add michael-gentile.webp.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/data/GS-Investors.xlsx
+++ b/data/GS-Investors.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="587" uniqueCount="252">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="633" uniqueCount="256">
   <si>
     <t xml:space="preserve">investor</t>
   </si>
@@ -745,6 +745,9 @@
     <t xml:space="preserve">Jon Binder</t>
   </si>
   <si>
+    <t xml:space="preserve">GS founder</t>
+  </si>
+  <si>
     <t xml:space="preserve">David Erfle</t>
   </si>
   <si>
@@ -772,10 +775,19 @@
     <t xml:space="preserve">Peter Krauth </t>
   </si>
   <si>
+    <t xml:space="preserve">silver bull</t>
+  </si>
+  <si>
     <t xml:space="preserve">Lundin Family</t>
   </si>
   <si>
+    <t xml:space="preserve">Jack and Adam Lundin </t>
+  </si>
+  <si>
     <t xml:space="preserve">Michael Gentile </t>
+  </si>
+  <si>
+    <t xml:space="preserve">investment fund</t>
   </si>
 </sst>
 </file>
@@ -938,7 +950,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="41">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1075,7 +1087,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="10" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="10" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1083,7 +1095,23 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -3824,6 +3852,9 @@
       <c r="H80" s="33" t="n">
         <v>46191</v>
       </c>
+      <c r="I80" s="34" t="s">
+        <v>241</v>
+      </c>
     </row>
     <row r="81" s="34" customFormat="true" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="32" t="s">
@@ -3853,54 +3884,205 @@
     </row>
     <row r="82" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A82" s="35" t="s">
-        <v>241</v>
-      </c>
-      <c r="B82" s="0"/>
-      <c r="I82" s="1" t="s">
         <v>242</v>
+      </c>
+      <c r="B82" s="36" t="s">
+        <v>49</v>
+      </c>
+      <c r="C82" s="36" t="s">
+        <v>50</v>
+      </c>
+      <c r="D82" s="36" t="s">
+        <v>15</v>
+      </c>
+      <c r="E82" s="36" t="s">
+        <v>28</v>
+      </c>
+      <c r="F82" s="36" t="s">
+        <v>155</v>
+      </c>
+      <c r="G82" s="36" t="s">
+        <v>28</v>
+      </c>
+      <c r="H82" s="37" t="n">
+        <v>46191</v>
+      </c>
+      <c r="I82" s="38" t="s">
+        <v>243</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A83" s="35" t="s">
-        <v>243</v>
-      </c>
-      <c r="B83" s="0"/>
-      <c r="C83" s="0"/>
-      <c r="I83" s="1" t="s">
         <v>244</v>
       </c>
+      <c r="B83" s="36" t="s">
+        <v>49</v>
+      </c>
+      <c r="C83" s="36" t="s">
+        <v>50</v>
+      </c>
+      <c r="D83" s="36" t="s">
+        <v>15</v>
+      </c>
+      <c r="E83" s="36" t="s">
+        <v>28</v>
+      </c>
+      <c r="F83" s="36" t="s">
+        <v>155</v>
+      </c>
+      <c r="G83" s="36" t="s">
+        <v>28</v>
+      </c>
+      <c r="H83" s="37" t="n">
+        <v>46191</v>
+      </c>
+      <c r="I83" s="38" t="s">
+        <v>245</v>
+      </c>
     </row>
     <row r="84" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A84" s="36" t="s">
-        <v>245</v>
-      </c>
-      <c r="B84" s="0"/>
-      <c r="I84" s="36" t="s">
+      <c r="A84" s="39" t="s">
         <v>246</v>
       </c>
+      <c r="B84" s="36" t="s">
+        <v>49</v>
+      </c>
+      <c r="C84" s="36" t="s">
+        <v>50</v>
+      </c>
+      <c r="D84" s="36" t="s">
+        <v>15</v>
+      </c>
+      <c r="E84" s="36" t="s">
+        <v>28</v>
+      </c>
+      <c r="F84" s="36" t="s">
+        <v>155</v>
+      </c>
+      <c r="G84" s="36" t="s">
+        <v>28</v>
+      </c>
+      <c r="H84" s="37" t="n">
+        <v>46191</v>
+      </c>
+      <c r="I84" s="39" t="s">
+        <v>247</v>
+      </c>
     </row>
     <row r="85" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A85" s="1" t="s">
-        <v>247</v>
-      </c>
-      <c r="B85" s="0"/>
-      <c r="I85" s="1" t="s">
+      <c r="A85" s="38" t="s">
         <v>248</v>
       </c>
+      <c r="B85" s="36" t="s">
+        <v>49</v>
+      </c>
+      <c r="C85" s="36" t="s">
+        <v>50</v>
+      </c>
+      <c r="D85" s="36" t="s">
+        <v>15</v>
+      </c>
+      <c r="E85" s="36" t="s">
+        <v>28</v>
+      </c>
+      <c r="F85" s="36" t="s">
+        <v>155</v>
+      </c>
+      <c r="G85" s="36" t="s">
+        <v>28</v>
+      </c>
+      <c r="H85" s="37" t="n">
+        <v>46191</v>
+      </c>
+      <c r="I85" s="38" t="s">
+        <v>249</v>
+      </c>
     </row>
     <row r="86" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A86" s="1" t="s">
-        <v>249</v>
+      <c r="A86" s="38" t="s">
+        <v>250</v>
+      </c>
+      <c r="B86" s="36" t="s">
+        <v>49</v>
+      </c>
+      <c r="C86" s="36" t="s">
+        <v>50</v>
+      </c>
+      <c r="D86" s="36" t="s">
+        <v>15</v>
+      </c>
+      <c r="E86" s="36" t="s">
+        <v>28</v>
+      </c>
+      <c r="F86" s="36" t="s">
+        <v>155</v>
+      </c>
+      <c r="G86" s="36" t="s">
+        <v>28</v>
+      </c>
+      <c r="H86" s="37" t="n">
+        <v>46191</v>
+      </c>
+      <c r="I86" s="40" t="s">
+        <v>251</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A87" s="1" t="s">
-        <v>250</v>
+      <c r="A87" s="38" t="s">
+        <v>252</v>
+      </c>
+      <c r="B87" s="36" t="s">
+        <v>49</v>
+      </c>
+      <c r="C87" s="36" t="s">
+        <v>50</v>
+      </c>
+      <c r="D87" s="36" t="s">
+        <v>15</v>
+      </c>
+      <c r="E87" s="36" t="s">
+        <v>28</v>
+      </c>
+      <c r="F87" s="36" t="s">
+        <v>155</v>
+      </c>
+      <c r="G87" s="36" t="s">
+        <v>28</v>
+      </c>
+      <c r="H87" s="37" t="n">
+        <v>46191</v>
+      </c>
+      <c r="I87" s="40" t="s">
+        <v>253</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A88" s="36" t="s">
-        <v>251</v>
+      <c r="A88" s="39" t="s">
+        <v>254</v>
+      </c>
+      <c r="B88" s="36" t="s">
+        <v>49</v>
+      </c>
+      <c r="C88" s="36" t="s">
+        <v>50</v>
+      </c>
+      <c r="D88" s="36" t="s">
+        <v>15</v>
+      </c>
+      <c r="E88" s="36" t="s">
+        <v>28</v>
+      </c>
+      <c r="F88" s="36" t="s">
+        <v>155</v>
+      </c>
+      <c r="G88" s="36" t="s">
+        <v>28</v>
+      </c>
+      <c r="H88" s="37" t="n">
+        <v>46191</v>
+      </c>
+      <c r="I88" s="40" t="s">
+        <v>255</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Sync investor workbook: add Nomi Prins and refresh positions
Update GS-Investors.xlsx (19 investors, 88 position rows) and regenerated investors.json after investors:sync.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/data/GS-Investors.xlsx
+++ b/data/GS-Investors.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="633" uniqueCount="256">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="641" uniqueCount="258">
   <si>
     <t xml:space="preserve">investor</t>
   </si>
@@ -787,7 +787,13 @@
     <t xml:space="preserve">Michael Gentile </t>
   </si>
   <si>
-    <t xml:space="preserve">investment fund</t>
+    <t xml:space="preserve">investment fund manager</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nomi Prins</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nomi Prins is a geopolitical financial expert and financial historian who sheds light on the dark corners of the global economy </t>
   </si>
 </sst>
 </file>
@@ -801,7 +807,7 @@
     <numFmt numFmtId="167" formatCode="yyyy\-m"/>
     <numFmt numFmtId="168" formatCode="m/d/yyyy"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="7">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -846,12 +852,6 @@
       <name val="Cambria"/>
       <family val="0"/>
       <charset val="1"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FF000000"/>
-      <name val="Arial"/>
-      <family val="0"/>
     </font>
   </fonts>
   <fills count="11">
@@ -950,7 +950,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="38">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1063,15 +1063,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="9" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="5" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="7" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="9" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1087,11 +1079,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="10" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="10" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1107,12 +1099,8 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -1376,7 +1364,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="19.38"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="23.75"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="22.75"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="88.52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="88.52"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3645,7 +3633,7 @@
         <v>46143</v>
       </c>
     </row>
-    <row r="73" s="29" customFormat="true" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="73" s="14" customFormat="true" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="12" t="s">
         <v>208</v>
       </c>
@@ -3671,7 +3659,7 @@
         <v>46153</v>
       </c>
     </row>
-    <row r="74" s="29" customFormat="true" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="74" s="14" customFormat="true" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="12" t="s">
         <v>208</v>
       </c>
@@ -3697,7 +3685,7 @@
         <v>46153</v>
       </c>
     </row>
-    <row r="75" s="29" customFormat="true" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="75" s="14" customFormat="true" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="12" t="s">
         <v>208</v>
       </c>
@@ -3723,7 +3711,7 @@
         <v>46153</v>
       </c>
     </row>
-    <row r="76" s="30" customFormat="true" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="76" s="22" customFormat="true" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="21" t="s">
         <v>218</v>
       </c>
@@ -3749,7 +3737,7 @@
         <v>2025</v>
       </c>
     </row>
-    <row r="77" s="30" customFormat="true" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="77" s="22" customFormat="true" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="21" t="s">
         <v>218</v>
       </c>
@@ -3771,11 +3759,11 @@
       <c r="G77" s="21" t="s">
         <v>228</v>
       </c>
-      <c r="H77" s="31" t="n">
+      <c r="H77" s="29" t="n">
         <v>45362</v>
       </c>
     </row>
-    <row r="78" s="30" customFormat="true" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="78" s="22" customFormat="true" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="21" t="s">
         <v>218</v>
       </c>
@@ -3801,7 +3789,7 @@
         <v>2024</v>
       </c>
     </row>
-    <row r="79" s="30" customFormat="true" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="79" s="22" customFormat="true" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="21" t="s">
         <v>218</v>
       </c>
@@ -3823,270 +3811,296 @@
       <c r="G79" s="21" t="s">
         <v>239</v>
       </c>
-      <c r="H79" s="31" t="n">
+      <c r="H79" s="29" t="n">
         <v>45981</v>
       </c>
     </row>
-    <row r="80" s="34" customFormat="true" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A80" s="32" t="s">
+    <row r="80" s="32" customFormat="true" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A80" s="30" t="s">
         <v>240</v>
       </c>
-      <c r="B80" s="32" t="s">
+      <c r="B80" s="30" t="s">
         <v>153</v>
       </c>
-      <c r="C80" s="32" t="s">
+      <c r="C80" s="30" t="s">
         <v>154</v>
       </c>
-      <c r="D80" s="32" t="s">
-        <v>15</v>
-      </c>
-      <c r="E80" s="32" t="s">
-        <v>28</v>
-      </c>
-      <c r="F80" s="32" t="s">
+      <c r="D80" s="30" t="s">
+        <v>15</v>
+      </c>
+      <c r="E80" s="30" t="s">
+        <v>28</v>
+      </c>
+      <c r="F80" s="30" t="s">
         <v>155</v>
       </c>
-      <c r="G80" s="32" t="s">
-        <v>28</v>
-      </c>
-      <c r="H80" s="33" t="n">
+      <c r="G80" s="30" t="s">
+        <v>28</v>
+      </c>
+      <c r="H80" s="31" t="n">
         <v>46191</v>
       </c>
-      <c r="I80" s="34" t="s">
+      <c r="I80" s="32" t="s">
         <v>241</v>
       </c>
     </row>
-    <row r="81" s="34" customFormat="true" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A81" s="32" t="s">
+    <row r="81" s="32" customFormat="true" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A81" s="30" t="s">
         <v>240</v>
       </c>
-      <c r="B81" s="32" t="s">
+      <c r="B81" s="30" t="s">
         <v>49</v>
       </c>
-      <c r="C81" s="32" t="s">
+      <c r="C81" s="30" t="s">
         <v>50</v>
       </c>
-      <c r="D81" s="32" t="s">
-        <v>15</v>
-      </c>
-      <c r="E81" s="32" t="s">
-        <v>28</v>
-      </c>
-      <c r="F81" s="32" t="s">
+      <c r="D81" s="30" t="s">
+        <v>15</v>
+      </c>
+      <c r="E81" s="30" t="s">
+        <v>28</v>
+      </c>
+      <c r="F81" s="30" t="s">
         <v>155</v>
       </c>
-      <c r="G81" s="32" t="s">
-        <v>28</v>
-      </c>
-      <c r="H81" s="33" t="n">
+      <c r="G81" s="30" t="s">
+        <v>28</v>
+      </c>
+      <c r="H81" s="31" t="n">
         <v>46191</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A82" s="35" t="s">
+      <c r="A82" s="33" t="s">
         <v>242</v>
       </c>
-      <c r="B82" s="36" t="s">
+      <c r="B82" s="34" t="s">
         <v>49</v>
       </c>
-      <c r="C82" s="36" t="s">
+      <c r="C82" s="34" t="s">
         <v>50</v>
       </c>
-      <c r="D82" s="36" t="s">
-        <v>15</v>
-      </c>
-      <c r="E82" s="36" t="s">
-        <v>28</v>
-      </c>
-      <c r="F82" s="36" t="s">
+      <c r="D82" s="34" t="s">
+        <v>15</v>
+      </c>
+      <c r="E82" s="34" t="s">
+        <v>28</v>
+      </c>
+      <c r="F82" s="34" t="s">
         <v>155</v>
       </c>
-      <c r="G82" s="36" t="s">
-        <v>28</v>
-      </c>
-      <c r="H82" s="37" t="n">
+      <c r="G82" s="34" t="s">
+        <v>28</v>
+      </c>
+      <c r="H82" s="35" t="n">
         <v>46191</v>
       </c>
-      <c r="I82" s="38" t="s">
+      <c r="I82" s="36" t="s">
         <v>243</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A83" s="35" t="s">
+      <c r="A83" s="33" t="s">
         <v>244</v>
       </c>
-      <c r="B83" s="36" t="s">
+      <c r="B83" s="34" t="s">
         <v>49</v>
       </c>
-      <c r="C83" s="36" t="s">
+      <c r="C83" s="34" t="s">
         <v>50</v>
       </c>
-      <c r="D83" s="36" t="s">
-        <v>15</v>
-      </c>
-      <c r="E83" s="36" t="s">
-        <v>28</v>
-      </c>
-      <c r="F83" s="36" t="s">
+      <c r="D83" s="34" t="s">
+        <v>15</v>
+      </c>
+      <c r="E83" s="34" t="s">
+        <v>28</v>
+      </c>
+      <c r="F83" s="34" t="s">
         <v>155</v>
       </c>
-      <c r="G83" s="36" t="s">
-        <v>28</v>
-      </c>
-      <c r="H83" s="37" t="n">
+      <c r="G83" s="34" t="s">
+        <v>28</v>
+      </c>
+      <c r="H83" s="35" t="n">
         <v>46191</v>
       </c>
-      <c r="I83" s="38" t="s">
+      <c r="I83" s="36" t="s">
         <v>245</v>
       </c>
     </row>
     <row r="84" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A84" s="39" t="s">
+      <c r="A84" s="36" t="s">
         <v>246</v>
       </c>
-      <c r="B84" s="36" t="s">
+      <c r="B84" s="34" t="s">
         <v>49</v>
       </c>
-      <c r="C84" s="36" t="s">
+      <c r="C84" s="34" t="s">
         <v>50</v>
       </c>
-      <c r="D84" s="36" t="s">
-        <v>15</v>
-      </c>
-      <c r="E84" s="36" t="s">
-        <v>28</v>
-      </c>
-      <c r="F84" s="36" t="s">
+      <c r="D84" s="34" t="s">
+        <v>15</v>
+      </c>
+      <c r="E84" s="34" t="s">
+        <v>28</v>
+      </c>
+      <c r="F84" s="34" t="s">
         <v>155</v>
       </c>
-      <c r="G84" s="36" t="s">
-        <v>28</v>
-      </c>
-      <c r="H84" s="37" t="n">
+      <c r="G84" s="34" t="s">
+        <v>28</v>
+      </c>
+      <c r="H84" s="35" t="n">
         <v>46191</v>
       </c>
-      <c r="I84" s="39" t="s">
+      <c r="I84" s="36" t="s">
         <v>247</v>
       </c>
     </row>
     <row r="85" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A85" s="38" t="s">
+      <c r="A85" s="36" t="s">
         <v>248</v>
       </c>
-      <c r="B85" s="36" t="s">
+      <c r="B85" s="34" t="s">
         <v>49</v>
       </c>
-      <c r="C85" s="36" t="s">
+      <c r="C85" s="34" t="s">
         <v>50</v>
       </c>
-      <c r="D85" s="36" t="s">
-        <v>15</v>
-      </c>
-      <c r="E85" s="36" t="s">
-        <v>28</v>
-      </c>
-      <c r="F85" s="36" t="s">
+      <c r="D85" s="34" t="s">
+        <v>15</v>
+      </c>
+      <c r="E85" s="34" t="s">
+        <v>28</v>
+      </c>
+      <c r="F85" s="34" t="s">
         <v>155</v>
       </c>
-      <c r="G85" s="36" t="s">
-        <v>28</v>
-      </c>
-      <c r="H85" s="37" t="n">
+      <c r="G85" s="34" t="s">
+        <v>28</v>
+      </c>
+      <c r="H85" s="35" t="n">
         <v>46191</v>
       </c>
-      <c r="I85" s="38" t="s">
+      <c r="I85" s="36" t="s">
         <v>249</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A86" s="38" t="s">
+      <c r="A86" s="36" t="s">
         <v>250</v>
       </c>
-      <c r="B86" s="36" t="s">
+      <c r="B86" s="34" t="s">
         <v>49</v>
       </c>
-      <c r="C86" s="36" t="s">
+      <c r="C86" s="34" t="s">
         <v>50</v>
       </c>
-      <c r="D86" s="36" t="s">
-        <v>15</v>
-      </c>
-      <c r="E86" s="36" t="s">
-        <v>28</v>
-      </c>
-      <c r="F86" s="36" t="s">
+      <c r="D86" s="34" t="s">
+        <v>15</v>
+      </c>
+      <c r="E86" s="34" t="s">
+        <v>28</v>
+      </c>
+      <c r="F86" s="34" t="s">
         <v>155</v>
       </c>
-      <c r="G86" s="36" t="s">
-        <v>28</v>
-      </c>
-      <c r="H86" s="37" t="n">
+      <c r="G86" s="34" t="s">
+        <v>28</v>
+      </c>
+      <c r="H86" s="35" t="n">
         <v>46191</v>
       </c>
-      <c r="I86" s="40" t="s">
+      <c r="I86" s="36" t="s">
         <v>251</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A87" s="38" t="s">
+      <c r="A87" s="36" t="s">
         <v>252</v>
       </c>
-      <c r="B87" s="36" t="s">
+      <c r="B87" s="34" t="s">
         <v>49</v>
       </c>
-      <c r="C87" s="36" t="s">
+      <c r="C87" s="34" t="s">
         <v>50</v>
       </c>
-      <c r="D87" s="36" t="s">
-        <v>15</v>
-      </c>
-      <c r="E87" s="36" t="s">
-        <v>28</v>
-      </c>
-      <c r="F87" s="36" t="s">
+      <c r="D87" s="34" t="s">
+        <v>15</v>
+      </c>
+      <c r="E87" s="34" t="s">
+        <v>28</v>
+      </c>
+      <c r="F87" s="34" t="s">
         <v>155</v>
       </c>
-      <c r="G87" s="36" t="s">
-        <v>28</v>
-      </c>
-      <c r="H87" s="37" t="n">
+      <c r="G87" s="34" t="s">
+        <v>28</v>
+      </c>
+      <c r="H87" s="35" t="n">
         <v>46191</v>
       </c>
-      <c r="I87" s="40" t="s">
+      <c r="I87" s="36" t="s">
         <v>253</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A88" s="39" t="s">
+      <c r="A88" s="36" t="s">
         <v>254</v>
       </c>
-      <c r="B88" s="36" t="s">
+      <c r="B88" s="34" t="s">
         <v>49</v>
       </c>
-      <c r="C88" s="36" t="s">
+      <c r="C88" s="34" t="s">
         <v>50</v>
       </c>
-      <c r="D88" s="36" t="s">
-        <v>15</v>
-      </c>
-      <c r="E88" s="36" t="s">
-        <v>28</v>
-      </c>
-      <c r="F88" s="36" t="s">
+      <c r="D88" s="34" t="s">
+        <v>15</v>
+      </c>
+      <c r="E88" s="34" t="s">
+        <v>28</v>
+      </c>
+      <c r="F88" s="34" t="s">
         <v>155</v>
       </c>
-      <c r="G88" s="36" t="s">
-        <v>28</v>
-      </c>
-      <c r="H88" s="37" t="n">
+      <c r="G88" s="34" t="s">
+        <v>28</v>
+      </c>
+      <c r="H88" s="35" t="n">
         <v>46191</v>
       </c>
-      <c r="I88" s="40" t="s">
+      <c r="I88" s="36" t="s">
         <v>255</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A89" s="0"/>
+      <c r="A89" s="36" t="s">
+        <v>256</v>
+      </c>
+      <c r="B89" s="34" t="s">
+        <v>49</v>
+      </c>
+      <c r="C89" s="34" t="s">
+        <v>50</v>
+      </c>
+      <c r="D89" s="34" t="s">
+        <v>15</v>
+      </c>
+      <c r="E89" s="34" t="s">
+        <v>28</v>
+      </c>
+      <c r="F89" s="34" t="s">
+        <v>155</v>
+      </c>
+      <c r="G89" s="34" t="s">
+        <v>28</v>
+      </c>
+      <c r="H89" s="35" t="n">
+        <v>46191</v>
+      </c>
+      <c r="I89" s="37" t="s">
+        <v>257</v>
+      </c>
     </row>
     <row r="1048573" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="1048574" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>

</xml_diff>